<commit_message>
stats and graph updates
</commit_message>
<xml_diff>
--- a/trichomes.xlsx
+++ b/trichomes.xlsx
@@ -8,12 +8,12 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\oia08\Documents\GitHub\Kjuka_MasterThesis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7EACF78F-FC45-400A-BF18-964A65EE49F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{A89D3BA6-0F03-4741-95C1-F6E9B6456DF4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{56149024-E4D2-428E-8250-EC47EDC159A8}"/>
+    <workbookView xWindow="-28920" yWindow="-105" windowWidth="29040" windowHeight="15720" xr2:uid="{56149024-E4D2-428E-8250-EC47EDC159A8}"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="trichomes" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="320" uniqueCount="52">
   <si>
     <t>Treatment</t>
   </si>
@@ -173,12 +173,6 @@
     <t>Plant_ID</t>
   </si>
   <si>
-    <t>Atharvest</t>
-  </si>
-  <si>
-    <t>Beforeharvest</t>
-  </si>
-  <si>
     <t>No Beetle</t>
   </si>
   <si>
@@ -186,13 +180,25 @@
   </si>
   <si>
     <t>Microplastic,</t>
+  </si>
+  <si>
+    <t>Harvest</t>
+  </si>
+  <si>
+    <t>Week 15</t>
+  </si>
+  <si>
+    <t>At Harvest</t>
+  </si>
+  <si>
+    <t>Trichome_count</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -205,6 +211,12 @@
       <color rgb="FF000000"/>
       <name val="Calibri"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -564,8 +576,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{31BDA673-B9C8-49E9-B438-D5C3874811A2}">
-  <dimension ref="A1:I43"/>
+  <dimension ref="A1:I85"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="6" max="6" width="10" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
@@ -578,731 +593,1469 @@
         <v>44</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>45</v>
-      </c>
+        <v>51</v>
+      </c>
+      <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C2" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E2">
         <v>85</v>
-      </c>
-      <c r="E2">
-        <v>69</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="D3">
-        <v>121</v>
+        <v>45</v>
+      </c>
+      <c r="C3" t="str">
+        <f>C2</f>
+        <v>C-Sb-1</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E3">
-        <v>104</v>
+        <v>69</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="D4">
-        <v>86</v>
+        <v>3</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="E4">
-        <v>32</v>
+        <v>121</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="D5">
-        <v>105</v>
+        <v>45</v>
+      </c>
+      <c r="C5" t="str">
+        <f>C4</f>
+        <v>C-Sb-2</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E5">
-        <v>168</v>
+        <v>104</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6">
-        <v>77</v>
+        <v>4</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="E6">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="D7">
-        <v>46</v>
+        <v>45</v>
+      </c>
+      <c r="C7" t="str">
+        <f>C6</f>
+        <v>C-Sb-3</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E7">
-        <v>103</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="D8">
-        <v>78</v>
+        <v>5</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="E8">
-        <v>106</v>
-      </c>
-      <c r="F8" s="1"/>
+        <v>105</v>
+      </c>
       <c r="G8" s="1"/>
       <c r="H8" s="1"/>
       <c r="I8" s="1"/>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="D9">
-        <v>62</v>
+        <v>45</v>
+      </c>
+      <c r="C9" t="str">
+        <f>C8</f>
+        <v>C-Sb-4</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E9">
-        <v>73</v>
+        <v>168</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10">
-        <v>154</v>
+        <v>6</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="E10">
-        <v>91</v>
+        <v>77</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C11" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="D11">
-        <v>167</v>
+        <v>45</v>
+      </c>
+      <c r="C11" t="str">
+        <f>C10</f>
+        <v>C-Sb-5</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E11">
-        <v>113</v>
+        <v>85</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D12">
-        <v>76</v>
+        <v>7</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="E12">
-        <v>62</v>
+        <v>46</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="D13">
-        <v>118</v>
+        <v>45</v>
+      </c>
+      <c r="C13" t="str">
+        <f>C12</f>
+        <v>C-Sb-6</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E13">
-        <v>92</v>
+        <v>103</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="D14">
-        <v>65</v>
+        <v>8</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="E14">
-        <v>68</v>
+        <v>78</v>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C15" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="D15">
-        <v>83</v>
+        <v>45</v>
+      </c>
+      <c r="C15" t="str">
+        <f>C14</f>
+        <v>C-Sb-7</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E15">
-        <v>83</v>
+        <v>106</v>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>1</v>
+        <v>45</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="D16">
-        <v>56</v>
+        <v>9</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="E16">
-        <v>104</v>
+        <v>62</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C17" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="D17">
-        <v>96</v>
+        <v>45</v>
+      </c>
+      <c r="C17" t="str">
+        <f>C16</f>
+        <v>C-Sb-8</v>
+      </c>
+      <c r="D17" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E17">
-        <v>71</v>
+        <v>73</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="D18">
-        <v>184</v>
+        <v>10</v>
+      </c>
+      <c r="D18" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="E18">
-        <v>153</v>
+        <v>154</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C19" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="D19">
-        <v>123</v>
+        <v>1</v>
+      </c>
+      <c r="C19" t="str">
+        <f>C18</f>
+        <v>C-MBB-1</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E19">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D20">
-        <v>99</v>
+        <v>11</v>
+      </c>
+      <c r="D20" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="E20">
-        <v>121</v>
+        <v>167</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D21">
-        <v>92</v>
+        <v>1</v>
+      </c>
+      <c r="C21" t="str">
+        <f>C20</f>
+        <v>C-MBB-2</v>
+      </c>
+      <c r="D21" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E21">
-        <v>106</v>
+        <v>113</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D22">
-        <v>99</v>
+        <v>12</v>
+      </c>
+      <c r="D22" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="E22">
-        <v>111</v>
+        <v>76</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C23" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D23">
-        <v>131</v>
+        <v>1</v>
+      </c>
+      <c r="C23" t="str">
+        <f>C22</f>
+        <v>C-MBB-3</v>
+      </c>
+      <c r="D23" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E23">
-        <v>116</v>
+        <v>62</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D24">
-        <v>62</v>
+        <v>13</v>
+      </c>
+      <c r="D24" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="E24">
-        <v>96</v>
+        <v>118</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C25" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D25">
-        <v>93</v>
+        <v>1</v>
+      </c>
+      <c r="C25" t="str">
+        <f>C24</f>
+        <v>C-MBB-4</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E25">
-        <v>62</v>
+        <v>92</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D26">
-        <v>91</v>
+        <v>14</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="E26">
-        <v>95</v>
+        <v>65</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C27" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D27">
-        <v>102</v>
+        <v>1</v>
+      </c>
+      <c r="C27" t="str">
+        <f>C26</f>
+        <v>C-MBB-5</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E27">
-        <v>85</v>
+        <v>68</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="D28">
-        <v>107</v>
+        <v>15</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="E28">
-        <v>161</v>
+        <v>83</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C29" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="D29">
-        <v>80</v>
+        <v>1</v>
+      </c>
+      <c r="C29" t="str">
+        <f>C28</f>
+        <v>C-MBB-6</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E29">
-        <v>115</v>
+        <v>83</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>47</v>
+        <v>1</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D30">
-        <v>123</v>
+        <v>16</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>49</v>
       </c>
       <c r="E30">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C31" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="D31">
-        <v>61</v>
+      <c r="C31" t="str">
+        <f>C30</f>
+        <v>C-MBB-7</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>50</v>
       </c>
       <c r="E31">
-        <v>98</v>
+        <v>104</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C32" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E32">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A33" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B33" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C33" t="str">
+        <f>C32</f>
+        <v>C-MBB-8</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E33">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A34" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E34">
+        <v>184</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A35" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C35" t="str">
+        <f>C34</f>
+        <v>C-Ex-1</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E35">
+        <v>153</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A36" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B36" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E36">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A37" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B37" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C37" t="str">
+        <f>C36</f>
+        <v>C-Ex-2</v>
+      </c>
+      <c r="D37" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E37">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A38" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B38" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E38">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A39" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C39" t="str">
+        <f>C38</f>
+        <v>C-Ex-3</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E39">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A40" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D40" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E40">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A41" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B41" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C41" t="str">
+        <f>C40</f>
+        <v>C-Ex-4</v>
+      </c>
+      <c r="D41" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E41">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A42" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B42" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D42" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E42">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A43" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="B43" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C43" t="str">
+        <f>C42</f>
+        <v>C-Ex-5</v>
+      </c>
+      <c r="D43" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E43">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A44" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B44" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C44" t="s">
+        <v>23</v>
+      </c>
+      <c r="D44" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E44">
+        <v>131</v>
+      </c>
+      <c r="F44" s="1"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A45" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B45" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C45" t="s">
+        <v>23</v>
+      </c>
+      <c r="D45" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E45">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A46" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B46" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C46" t="s">
+        <v>24</v>
+      </c>
+      <c r="D46" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E46">
+        <v>62</v>
+      </c>
+      <c r="F46" s="1"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A47" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B47" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C47" t="s">
+        <v>24</v>
+      </c>
+      <c r="D47" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E47">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A48" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B48" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="D48" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E48">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A49" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C49" t="s">
+        <v>25</v>
+      </c>
+      <c r="D49" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E49">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="50" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B50" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D50" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E50">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="51" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A51" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B51" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C51" t="s">
+        <v>26</v>
+      </c>
+      <c r="D51" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E51">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="52" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A52" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B52" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="D52" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E52">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="53" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A53" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B53" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C53" t="s">
+        <v>27</v>
+      </c>
+      <c r="D53" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E53">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A54" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="D54" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E54">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="55" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A55" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B55" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C55" t="s">
+        <v>28</v>
+      </c>
+      <c r="D55" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E55">
+        <v>161</v>
+      </c>
+    </row>
+    <row r="56" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B56" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="D56" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E56">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="57" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A57" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B57" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C57" t="s">
+        <v>29</v>
+      </c>
+      <c r="D57" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E57">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="58" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A58" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B58" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="D58" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E58">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="59" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A59" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B59" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C59" t="s">
+        <v>30</v>
+      </c>
+      <c r="D59" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E59">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="60" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A60" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B60" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="D60" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E60">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="61" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A61" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B61" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C61" t="s">
+        <v>31</v>
+      </c>
+      <c r="D61" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E61">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="62" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A62" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B62" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C62" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="D32">
+      <c r="D62" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E62">
         <v>89</v>
       </c>
-      <c r="E32">
+    </row>
+    <row r="63" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A63" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B63" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C63" t="s">
+        <v>32</v>
+      </c>
+      <c r="D63" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E63">
         <v>147</v>
       </c>
     </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A33" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B33" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C33" s="1" t="s">
+    <row r="64" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A64" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C64" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="D33">
+      <c r="D64" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E64">
         <v>127</v>
       </c>
-      <c r="E33">
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A65" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C65" t="s">
+        <v>33</v>
+      </c>
+      <c r="D65" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E65">
         <v>103</v>
       </c>
     </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A34" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B34" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C34" s="1" t="s">
+    <row r="66" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C66" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="D34">
+      <c r="D66" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E66">
         <v>86</v>
       </c>
-      <c r="E34">
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A67" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C67" t="s">
+        <v>34</v>
+      </c>
+      <c r="D67" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E67">
         <v>111</v>
       </c>
     </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C35" s="1" t="s">
+    <row r="68" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A68" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C68" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="D35">
+      <c r="D68" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E68">
         <v>69</v>
       </c>
-      <c r="E35">
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A69" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C69" t="s">
+        <v>35</v>
+      </c>
+      <c r="D69" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E69">
         <v>137</v>
       </c>
     </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A36" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C36" s="1" t="s">
+    <row r="70" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A70" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C70" s="1" t="s">
         <v>36</v>
       </c>
-      <c r="D36">
+      <c r="D70" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E70">
         <v>63</v>
       </c>
-      <c r="E36">
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A71" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C71" t="s">
+        <v>36</v>
+      </c>
+      <c r="D71" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E71">
         <v>85</v>
       </c>
     </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A37" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B37" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C37" s="1" t="s">
+    <row r="72" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A72" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C72" s="1" t="s">
         <v>37</v>
       </c>
-      <c r="D37">
+      <c r="D72" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E72">
         <v>90</v>
       </c>
-      <c r="E37">
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A73" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C73" t="s">
+        <v>37</v>
+      </c>
+      <c r="D73" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E73">
         <v>58</v>
       </c>
     </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A38" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B38" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C38" s="1" t="s">
+    <row r="74" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A74" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C74" s="1" t="s">
         <v>38</v>
       </c>
-      <c r="D38">
+      <c r="D74" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E74">
         <v>93</v>
       </c>
-      <c r="E38">
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A75" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C75" t="s">
+        <v>38</v>
+      </c>
+      <c r="D75" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E75">
         <v>113</v>
       </c>
     </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A39" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C39" s="1" t="s">
+    <row r="76" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A76" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B76" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C76" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="D39">
+      <c r="D76" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E76">
         <v>61</v>
       </c>
-      <c r="E39">
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A77" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C77" t="s">
+        <v>39</v>
+      </c>
+      <c r="D77" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E77">
         <v>77</v>
       </c>
     </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A40" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B40" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C40" s="1" t="s">
+    <row r="78" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A78" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C78" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D40">
+      <c r="D78" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E78">
         <v>278</v>
       </c>
-      <c r="E40">
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A79" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B79" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C79" t="s">
+        <v>40</v>
+      </c>
+      <c r="D79" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E79">
         <v>190</v>
       </c>
     </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A41" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B41" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C41" s="1" t="s">
+    <row r="80" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A80" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B80" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C80" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="D41">
+      <c r="D80" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E80">
         <v>66</v>
       </c>
-      <c r="E41">
+    </row>
+    <row r="81" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A81" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B81" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C81" t="s">
+        <v>41</v>
+      </c>
+      <c r="D81" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E81">
         <v>52</v>
       </c>
     </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A42" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B42" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C42" s="1" t="s">
+    <row r="82" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A82" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B82" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C82" s="1" t="s">
         <v>42</v>
       </c>
-      <c r="D42">
+      <c r="D82" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E82">
         <v>74</v>
       </c>
-      <c r="E42">
+    </row>
+    <row r="83" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A83" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B83" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C83" t="s">
+        <v>42</v>
+      </c>
+      <c r="D83" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E83">
         <v>125</v>
       </c>
     </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A43" s="1" t="s">
-        <v>49</v>
-      </c>
-      <c r="B43" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C43" s="1" t="s">
+    <row r="84" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A84" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B84" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C84" s="1" t="s">
         <v>43</v>
       </c>
-      <c r="D43">
+      <c r="D84" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="E84">
         <v>126</v>
       </c>
-      <c r="E43">
+    </row>
+    <row r="85" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A85" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="B85" s="1" t="s">
+        <v>45</v>
+      </c>
+      <c r="C85" t="s">
+        <v>43</v>
+      </c>
+      <c r="D85" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="E85">
         <v>109</v>
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>